<commit_message>
Legg til BSAI-investorer som mangler i investorlisten
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DcyyLDs44cBFfbPiNKsev9
</commit_message>
<xml_diff>
--- a/barricade/Barricade_investordatabaser_h2026.xlsx
+++ b/barricade/Barricade_investordatabaser_h2026.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investorer" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BSAI topp 15" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BSAI alle scorede" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forklaring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mangler i listen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forklaring" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -98,6 +99,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -249,6 +253,23 @@
     <tableColumn id="14" name="Nettside"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Mangler" displayName="Mangler" ref="A1:H23" headerRowCount="1">
+  <autoFilter ref="A1:H23"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Prioritet"/>
+    <tableColumn id="2" name="Investor"/>
+    <tableColumn id="3" name="Land"/>
+    <tableColumn id="4" name="Type"/>
+    <tableColumn id="5" name="Fase"/>
+    <tableColumn id="6" name="Relevante porteføljeselskaper"/>
+    <tableColumn id="7" name="Begrunnelse"/>
+    <tableColumn id="8" name="Nettside"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1"/>
 </table>
 </file>
 
@@ -55507,6 +55528,999 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Prioritet</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Fase</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Relevante porteføljeselskaper</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Begrunnelse</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Nettside</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pi Labs</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Accelerator, Venture Capital</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Plentific, Propster, Qualis Flow</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Investerer bare i bygg og eiendom, fra pre-seed til serie A. Det mest segmentspesifikke fondet i BSAI.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>www.pilabs.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Seed Capital</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Proper</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Danmarks største seed-fond med nordisk mandat. Fund V la til resiliens.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>www.seedcapital.dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Ferd</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Family Investment Office, Venture Capital</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Norsk family office med VC-arm som er aktiv i proptech. Matcher investortype nr. 1 i søkeordanalysen.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>www.ferd.no</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>BitStone Capital</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Architrave, aedifion, Upmin</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Seed-fond kun for eiendoms- og byggteknologi.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>www.bitstone.capital/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>APX</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>promiseQ</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Har investert i AI-verifisering av videoalarmer for alarmmottak. Inntil 0,5 mill. EUR før serie A.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>apx.vc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Adara Ventures</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Intelex Vision</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Deeptech i Spania, Portugal, Frankrike og UK. AI-videoanalyse for sikkerhet i porteføljen. Relevant for Spania.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>www.adara.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Høy</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Acurio Ventures</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Intelex Vision</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Spansk VC med sikkerhetsrelevant portefølje. Relevant for Spania.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>www.acurio.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Swisscom Ventures</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Convertible Note, Early Stage Venture, Late Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>viboo, Deepomatic</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Telekom-CVC med investeringer i smarte bygg. Telekom passer som distribusjons- og SIM-partner.</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>ventures.swisscom.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Verve Ventures</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Locatee, Veesion</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Har investert i arbeidsplassanalyse og AI-videoovervåkning.</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>verve.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Chalmers Ventures AB</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Parakey</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Mobil adgangskontroll, nesten Barricades segment. Krever i hovedsak Chalmers-tilknytning.</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>www.chalmersventures.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Triple Point Ventures</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Debt, Early Stage Venture, Late Stage Venture, Post-Ipo, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>SeeChange</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>UK tidligfase med sanntids videoanalyse i porteføljen.</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>www.triplepoint.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Amadeus Capital Partners</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Private Equity, Seed</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Pimloc</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Har investert i AI-anonymisering av CCTV-opptak.</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>amadeuscapital.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Fuel Ventures</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>SearchLand, Martello, Moverly</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>SaaS- og plattformfond med flere proptech-investeringer.</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>fuel.ventures/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Inveready</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Private Equity Firm, Venture Capital, Venture Debt</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Debt, Early Stage Venture, Private Equity, Secondary Market, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Intelex Vision, Ciudadela</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Spansk investor med sikkerhet og proptech i porteføljen. Del av PE-plattform, så sjekk mandat.</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>inveready.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Innovestor</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Private Equity Firm, Venture Capital</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Private Equity</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Amplifiles, CloEE</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Nordisk vekstinvestor med proptech og IoT i porteføljen.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>www.innovestorgroup.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Butterfly Ventures</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Convertible Note, Early Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Nordisk seed for hardware og software som jobber mot maskinvare.</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>butterfly.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Almi Invest</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Sveriges mest aktive tidligfaseinvestor. Krever selskap i Sverige.</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>www.almi.se/en/venture-capital/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Middels</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Vaekstfonden</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Proper</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Dansk statlig fond. Krever dansk tilknytning.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>www.vf.dk</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Lav</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2150</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Venture</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Urban tech, men første billett er 3-15 mill. EUR i serie A. Passer en senere runde.</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>2150.vc</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Lav</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>EQT Ventures</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Venture</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Luko, Buena</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Har investert i smarthusforsikring, men skriver store billetter.</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>eqtventures.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Lav</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Norrsken VC</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Venture Capital</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Late Stage Venture, Seed, Venture</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Predium, Boldr</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Impact-fond. Mandatet passer dårlig.</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>www.norrsken.org/norrskenvc</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Lav</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Katapult</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Accelerator, Venture Capital</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Early Stage Venture, Seed</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>ClevAir</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Klima-, hav- og agritech. Passer ikke.</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>katapult.vc</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -55555,7 +56569,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>